<commit_message>
🐛 Keep balance sign convention when removing abs()
Credit the payer with -amount and debit allocations with +amount, so
positive still means owed. Only the income fixture changes; drop the
unit tests in favour of the end-to-end income test.
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/custom_category_trip_8.xlsx
+++ b/tricount_extractor/tests/data/expected_results/custom_category_trip_8.xlsx
@@ -952,7 +952,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bob</t>
+          <t>Alice</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -965,7 +965,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Bob</t>
         </is>
       </c>
       <c r="C3" t="n">

</xml_diff>